<commit_message>
feat: add period applicability matrix and period-mode analysis groundwork
</commit_message>
<xml_diff>
--- a/config/ratio_analysis_rulebook.xlsx
+++ b/config/ratio_analysis_rulebook.xlsx
@@ -15,6 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="text_templates" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="statement_links" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="display_policy" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="period_applicability" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2613,4 +2614,212 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>rule_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>period_mode</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>match_type</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>match_value</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>applicability</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>enabled</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>sort_order</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>PA001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>monitor</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>indicator_id_contains</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>turnover</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>na</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>?????????????????????????????</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>PA002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>monitor</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>indicator_id</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>roe</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>na</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>?????ROE????????????????????????</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>PA003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>monitor</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>indicator_id_contains</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>gross_margin</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>caution</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>???????????????????????????????</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H4" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>PA999</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>monitor</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>applicable</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>?????????????</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" t="n">
+        <v>999</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>